<commit_message>
Added MD file with instructions to set-up unified testing device. Updated minSdk from 28 to 29 due to: Impending drop of support for major project libraries, Important system file and location security changes, Availability of virtual devices.
</commit_message>
<xml_diff>
--- a/Dokumentace/Nefunkcni_pozadavky_tankovani.xlsx
+++ b/Dokumentace/Nefunkcni_pozadavky_tankovani.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jirivavra/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Fueling_Management_Tool\Dokumentace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A9E0C77-74F3-1442-9A7E-7D7E530BF8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8903284-0BB7-4E6C-8654-1EC6A1FA9D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="32220" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nefunkční požadavky" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -203,7 +202,7 @@
     <t>Kompatibilita se systémem Android</t>
   </si>
   <si>
-    <t>Aplikace musí být plně funkční a vizuálně responzivní na mobilních zařízeních s operačním systémem Android 9.0 (API level 28) a novějším.</t>
+    <t>Aplikace musí být plně funkční a vizuálně responzivní na mobilních zařízeních s operačním systémem Android 10.0 (API level 29) a novějším.</t>
   </si>
 </sst>
 </file>
@@ -559,7 +558,7 @@
     <tabColor rgb="FF654D9B"/>
   </sheetPr>
   <dimension ref="A1:C38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>

</xml_diff>